<commit_message>
Refactor notebook-first workflow and update modeling pipeline
</commit_message>
<xml_diff>
--- a/app/data/raw/lotto_history_latest.xlsx
+++ b/app/data/raw/lotto_history_latest.xlsx
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1218"/>
+  <dimension ref="A1:L1223"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7.70703125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -54116,6 +54116,226 @@
         </is>
       </c>
     </row>
+    <row r="1219">
+      <c r="A1219" t="n">
+        <v>1218</v>
+      </c>
+      <c r="B1219" t="n">
+        <v>1218</v>
+      </c>
+      <c r="C1219" t="n">
+        <v>3</v>
+      </c>
+      <c r="D1219" t="n">
+        <v>28</v>
+      </c>
+      <c r="E1219" t="n">
+        <v>31</v>
+      </c>
+      <c r="F1219" t="n">
+        <v>32</v>
+      </c>
+      <c r="G1219" t="n">
+        <v>42</v>
+      </c>
+      <c r="H1219" t="n">
+        <v>45</v>
+      </c>
+      <c r="I1219" t="n">
+        <v>25</v>
+      </c>
+      <c r="J1219" t="inlineStr">
+        <is>
+          <t>1등</t>
+        </is>
+      </c>
+      <c r="K1219" t="inlineStr">
+        <is>
+          <t>18 명</t>
+        </is>
+      </c>
+      <c r="L1219" t="inlineStr">
+        <is>
+          <t>1,714,482,042 원</t>
+        </is>
+      </c>
+    </row>
+    <row r="1220">
+      <c r="A1220" t="n">
+        <v>1219</v>
+      </c>
+      <c r="B1220" t="n">
+        <v>1219</v>
+      </c>
+      <c r="C1220" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1220" t="n">
+        <v>2</v>
+      </c>
+      <c r="E1220" t="n">
+        <v>15</v>
+      </c>
+      <c r="F1220" t="n">
+        <v>28</v>
+      </c>
+      <c r="G1220" t="n">
+        <v>39</v>
+      </c>
+      <c r="H1220" t="n">
+        <v>45</v>
+      </c>
+      <c r="I1220" t="n">
+        <v>31</v>
+      </c>
+      <c r="J1220" t="inlineStr">
+        <is>
+          <t>1등</t>
+        </is>
+      </c>
+      <c r="K1220" t="inlineStr">
+        <is>
+          <t>12 명</t>
+        </is>
+      </c>
+      <c r="L1220" t="inlineStr">
+        <is>
+          <t>2,508,232,844 원</t>
+        </is>
+      </c>
+    </row>
+    <row r="1221">
+      <c r="A1221" t="n">
+        <v>1220</v>
+      </c>
+      <c r="B1221" t="n">
+        <v>1220</v>
+      </c>
+      <c r="C1221" t="n">
+        <v>2</v>
+      </c>
+      <c r="D1221" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1221" t="n">
+        <v>25</v>
+      </c>
+      <c r="F1221" t="n">
+        <v>28</v>
+      </c>
+      <c r="G1221" t="n">
+        <v>34</v>
+      </c>
+      <c r="H1221" t="n">
+        <v>43</v>
+      </c>
+      <c r="I1221" t="n">
+        <v>16</v>
+      </c>
+      <c r="J1221" t="inlineStr">
+        <is>
+          <t>1등</t>
+        </is>
+      </c>
+      <c r="K1221" t="inlineStr">
+        <is>
+          <t>14 명</t>
+        </is>
+      </c>
+      <c r="L1221" t="inlineStr">
+        <is>
+          <t>2,114,514,161 원</t>
+        </is>
+      </c>
+    </row>
+    <row r="1222">
+      <c r="A1222" t="n">
+        <v>1221</v>
+      </c>
+      <c r="B1222" t="n">
+        <v>1221</v>
+      </c>
+      <c r="C1222" t="n">
+        <v>6</v>
+      </c>
+      <c r="D1222" t="n">
+        <v>13</v>
+      </c>
+      <c r="E1222" t="n">
+        <v>18</v>
+      </c>
+      <c r="F1222" t="n">
+        <v>28</v>
+      </c>
+      <c r="G1222" t="n">
+        <v>30</v>
+      </c>
+      <c r="H1222" t="n">
+        <v>36</v>
+      </c>
+      <c r="I1222" t="n">
+        <v>9</v>
+      </c>
+      <c r="J1222" t="inlineStr">
+        <is>
+          <t>1등</t>
+        </is>
+      </c>
+      <c r="K1222" t="inlineStr">
+        <is>
+          <t>16 명</t>
+        </is>
+      </c>
+      <c r="L1222" t="inlineStr">
+        <is>
+          <t>1,830,801,165 원</t>
+        </is>
+      </c>
+    </row>
+    <row r="1223">
+      <c r="A1223" t="n">
+        <v>1222</v>
+      </c>
+      <c r="B1223" t="n">
+        <v>1222</v>
+      </c>
+      <c r="C1223" t="n">
+        <v>4</v>
+      </c>
+      <c r="D1223" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1223" t="n">
+        <v>17</v>
+      </c>
+      <c r="F1223" t="n">
+        <v>22</v>
+      </c>
+      <c r="G1223" t="n">
+        <v>32</v>
+      </c>
+      <c r="H1223" t="n">
+        <v>41</v>
+      </c>
+      <c r="I1223" t="n">
+        <v>34</v>
+      </c>
+      <c r="J1223" t="inlineStr">
+        <is>
+          <t>1등</t>
+        </is>
+      </c>
+      <c r="K1223" t="inlineStr">
+        <is>
+          <t>24 명</t>
+        </is>
+      </c>
+      <c r="L1223" t="inlineStr">
+        <is>
+          <t>1,202,986,844 원</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>